<commit_message>
feat(leads): add trading software stack mapping and product packaging matrix per firm
</commit_message>
<xml_diff>
--- a/leads/XPredictor_Institutional_Leads.xlsx
+++ b/leads/XPredictor_Institutional_Leads.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Institutional Leads Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cold Email Sequences" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign KPI Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Offer by Software" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cold Email Sequences" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign KPI Tracker" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,17 +40,17 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="000066CC"/>
       <sz val="9"/>
       <u val="single"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +67,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2FF"/>
         <bgColor rgb="00EEF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBEB"/>
+        <bgColor rgb="00FFFBEB"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,21 +126,32 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,21 +517,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="43" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
     <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -539,40 +560,55 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Supported Trading Software</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Software Archetype</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tailored Product Offer</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Key Executive / Decision Maker</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Target Title</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Contact Email</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Custom Demo Sandbox Link</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Cold Outreach Hook</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Cold Email Subject Line</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Outreach Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes / Next Step</t>
         </is>
@@ -597,42 +633,57 @@
           <t>Prague, Czechia / EU</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 4, MetaTrader 5, cTrader, DXtrade</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; Multi-Platform</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Turnkey Client Portal Iframe Widget + Native MT5 EA Indicator (.mq5)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Otakar Suffner / Marek Vasicek</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Head of Risk</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>partners@ftmo.com</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=ftmo</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Preventing challenge failures in low-vol chop &amp; protecting funded accounts from Max Daily DD spikes with Bayesian Cones</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>FTMO x XPredictor: Dynamic Max Drawdown &amp; Reality Cone Copilot for Evaluation Desks</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="N2" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Primary target - largest retail prop firm</t>
         </is>
@@ -657,42 +708,57 @@
           <t>Dubai, UAE</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, MetaTrader 5, MetaTrader 4, cTrader</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack (TradeLocker)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker Chart Webhook + Client Dashboard Risk Copilot Widget</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Abdullah Jayed / Syed Lateef</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Head of Operations</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>partnerships@fundednext.com</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=fundednext</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Stellar challenge pass rate stabilization and volatility boundary defense for funded traders</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>FundedNext Stellar Desk: AI Historical Regime Matching &amp; Risk Copilot</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>High viral community in MENA/Asia</t>
         </is>
@@ -717,42 +783,57 @@
           <t>Chicago, IL, USA</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Tradovate, NinjaTrader, TradingView, Quantower</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Futures Prop Stack (Tradovate / NT)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>TradingView Pine Script / Webhook + NinjaTrader C# Risk Copilot Indicator</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Michael Patak</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Founder</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>partners@topstep.com</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=topstep</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Futures Trading Combine volatility boundaries and zero-lookahead regime forecasting</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Topstep Combine: Empirical Volatility Envelopes for Futures Traders</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>US Futures dominance</t>
         </is>
@@ -777,42 +858,57 @@
           <t>Texas, USA</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Tradovate, NinjaTrader, Rithmic</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Futures Prop Stack (Rithmic / NT)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>NinjaTrader 8 C# Add-on + Tradovate Browser Risk Extension</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Darrell Martin</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>support@apextraderfunding.com</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=apex</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Trailing threshold drawdown defense during high-variance news releases (CPI/FOMC)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Apex Trader Funding: Trailing Threshold Risk Copilot via Hybrid AI Cones</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Massive US retail volume</t>
         </is>
@@ -837,42 +933,57 @@
           <t>London, UK</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 5, cTrader, Alpha Pro Platform (TradingView)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; Proprietary Web</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Direct WebTrader Iframe Component + Native MT5 EA Indicator</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>George Baker</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Head of Trading</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>info@alphacapitalgroup.uk</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=AlphaCapital</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Advanced market microstructure and resting liquidity depth integration for UK/EU challenge desks</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Alpha Capital Group: Proprietary AI Historical Twin Matching Suite</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>Strong institutional branding</t>
         </is>
@@ -897,42 +1008,57 @@
           <t>Dubai, UAE</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, cTrader, Match-Trader</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack (TradeLocker)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker &amp; cTrader Dashboard Web Widget + Signal API</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Khaled Ayesh</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>support@fundingpips.com</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=FundingPips</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>Ultra-fast scaling plan risk modeling and 2-step evaluation retention copilot</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Funding Pips x XPredictor: Proprietary Risk Sandbox for Active Challengers</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>Rapidly growing Dubai prop desk</t>
         </is>
@@ -957,42 +1083,57 @@
           <t>Dallas, TX / Prague</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>E8X (Custom TradingView Engine), Match-Trader, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Web Engine (E8X)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>E8X REST/WebSocket API Integration + Custom Web Component</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Dylan Elchami</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Founder</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>partners@e8markets.com</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=E8</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>Customizable drawdown scaling and Bayesian Reality Cone volatility analytics for E8 Track</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>E8 Markets: Institutional AI Volatility Boundaries for Evaluation Desks</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>Tech-forward userbase</t>
         </is>
@@ -1017,42 +1158,57 @@
           <t>London / Tel Aviv</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 5, cTrader</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; cTrader</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Native MT5 Indicator (.mq5) + cTrader cBot/Indicator (C#)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Gil Ben Hur</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>help@the5ers.com</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=The5ers</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>Hyper-growth career program risk stabilization and swing-trading historical regime verification</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>The 5%ers: Proprietary Multi-Horizon Volatility Envelopes for Funded Desks</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>Specialized in serious swing traders</t>
         </is>
@@ -1077,42 +1233,57 @@
           <t>Dallas, USA</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, DXtrade, Match-Trader, cTrader</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Unified Embeddable Web Widget for DXtrade &amp; TradeLocker Client Portal</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Matthew Leech</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>support@myfundedfx.com</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=MyFundedFX</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>One-click embeddable web trader risk copilot for MT5/DXTrade/cTrader challenges</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>MyFundedFX: Embeddable AI Pattern Search &amp; Reality Cone Terminal</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>Multiple front-end trading platforms</t>
         </is>
@@ -1137,42 +1308,57 @@
           <t>London, UK</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 5, cTrader</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; cTrader</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Native MT5 Indicator + cTrader C# Risk Copilot</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Daniel Martin</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Head of Trading</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>cti@citytradersimperium.com</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=CTI</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>Professional funded trader portfolio protection and empirical analogue matching</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>CTI Desk: Institutional Risk Copilot &amp; 50M+ Historical Regime Search</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="N11" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>High funded account longevity</t>
         </is>
@@ -1197,42 +1383,57 @@
           <t>Dubai / UK</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, Match-Trader, DXtrade, cTrader</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack (TradeLocker)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Guardian Protector API Extension + TradeLocker Chart Overlay</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Sean Bainbridge</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>support@blueguardian.com</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=BlueGuardian</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>Guardian Protector tool enhancement via real-time +2.1σ / -2.1σ Bayesian envelopes</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>Blue Guardian Protector: Enhancing Trader Discipline with AI Reality Cones</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>Focus on automated risk protection</t>
         </is>
@@ -1257,42 +1458,57 @@
           <t>Cyprus / EU</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader Ecosystem</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Native MT5 EA Indicator + Client Area Evaluation Risk Widget</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Trading Operations</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Head of Risk Management</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>support@fidelcrest.com</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Fidelcrest</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>Micro and Pro trader challenge retention in choppy currency and gold regimes</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Fidelcrest Pro Desks: Causal AI Regime Matching &amp; Volatility Prediction</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>EU established prop firm</t>
         </is>
@@ -1317,42 +1533,57 @@
           <t>London, UK</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader Ecosystem</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Native MT5 Indicator + Risk Assessment Web Portal</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Karim Yousfi</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>support@audacitycapital.co.uk</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Audacity</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>Funded trader program risk management copilot for London session institutional desks</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>Audacity Capital: Proprietary AI Risk Copilot for Funded Traders</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>London institutional presence</t>
         </is>
@@ -1377,42 +1608,57 @@
           <t>Spain / UAE</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, Match-Trader, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack &amp; MT5</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker / MT5 Dual Package (Web Widget + .mq5 Indicator)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Partnerships Desk</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Head of Strategic Growth</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>support@goatfundedtrader.com</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=GoatFunded</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>No time-limit evaluation retention and zero-lookahead historical pattern matching</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>Goat Funded Trader: Turnkey AI Reality Cone Sandbox for Challengers</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>High retail traffic</t>
         </is>
@@ -1437,42 +1683,57 @@
           <t>London, UK</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 4, MetaTrader 5, cTrader, DXtrade</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; Multi-Platform</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>cTrader / MT5 Indicator Package + Client Area Embed</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Simon M.</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>COO</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>support@fundedtradingplus.com</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=FundedTradingPlus</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>Experienced and Master trader scaling with institutional order depth profile analytics</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>Funded Trading Plus: Bayesian Probability Cones for Master Challengers</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="N16" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>High TrustPilot ratings</t>
         </is>
@@ -1497,42 +1758,57 @@
           <t>Austin, TX, USA</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, Match-Trader, DXtrade</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker Webhook &amp; Client Dashboard Risk Copilot</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Blake Morrow</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Co-Founder</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>support@smartproptrader.com</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=SmartPropTrader</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>Affordable evaluation conversion lift and multi-asset MT5 indicator integration</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>Smart Prop Trader: Turnkey AI Risk Sandbox &amp; Native MT5 Indicator</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="N17" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>US retail trader appeal</t>
         </is>
@@ -1557,42 +1833,57 @@
           <t>London, UK</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>TradeLocker, Match-Trader, cTrader</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Embeddable Web Component + cTrader C# Indicator</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Executive Desk</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Head of Partnerships</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>support@bespokefundingprogram.com</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=BespokeFunding</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>Classic and Rapid challenge volatility monitoring with empirical forward projections</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>Bespoke Funding: Empirical Volatility Boundaries for Challenge Desks</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="N18" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>Flexible evaluation models</t>
         </is>
@@ -1617,42 +1908,57 @@
           <t>Naples, FL, USA</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Match-Trader, DXtrade</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Modern Web Prop Stack</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Turnkey Client Portal Iframe Widget</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Jana Seaman</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>info@surgetrader.com</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=SurgeTrader</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
         <is>
           <t>Audition pass rate optimization and institutional Gold/Index regime modeling</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>SurgeTrader Audition Desk: AI Historical Analogue &amp; Risk Copilot</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="N19" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>Single-phase evaluation focus</t>
         </is>
@@ -1677,42 +1983,57 @@
           <t>Hungary / EU</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>cTrader, Match-Trader</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>cTrader &amp; Modern Web</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>cTrader C# Indicator + Web Dashboard Risk Widget</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Executive Team</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Head of Risk &amp; Trading</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>support@trueforexfunds.com</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=TrueForexFunds</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>Proprietary MT5 liquidity integration and dynamic cascade stress-testing</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>True Forex Funds: Proprietary AI Risk Copilot for Funded Desks</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="N20" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>European footprint</t>
         </is>
@@ -1737,42 +2058,57 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Tradovate, NinjaTrader</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Futures Prop Stack</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>NinjaTrader 8 C# Indicator + Tradovate Risk Overlay</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Bob Iaccino</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Head Trader &amp; Co-Founder</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>support@fasttracktrading.net</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="K21" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=FastTrack</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr">
         <is>
           <t>Immediate funding account protection and intraday volatility dispersion boundaries</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>Fast Track Trading: AI Volatility Cones for Direct Funded Accounts</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="N21" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="O21" s="3" t="inlineStr">
         <is>
           <t>Futures direct funding</t>
         </is>
@@ -1787,7 +2123,7 @@
           <t>IC Markets</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker (ECN)</t>
         </is>
@@ -1797,42 +2133,57 @@
           <t>Sydney, Australia / CySEC / FSA</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5, cTrader</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>TradingView Pine Script Tool + Native MT5 EA + Client Area Web Iframe</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Andrew Budzinski</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Managing Director</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>institutional@icmarkets.com</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=icmarkets</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>Client retention in chop &amp; boosting monthly lot turnover on Raw Spread ECN accounts via AI confidence metrics</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>IC Markets Client Area: Embeddable AI Reality Cone Terminal &amp; 18x Lot ROI</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="N22" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>World's largest FX/CFD volume broker</t>
         </is>
@@ -1847,7 +2198,7 @@
           <t>Pepperstone</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -1857,42 +2208,57 @@
           <t>Melbourne, Australia / FCA / CySEC</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5, cTrader</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>TradingView Integration + Client Area 'Razor AI' Embed + MT5 EA</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Tamas Szabo</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Group CEO</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>institutional@pepperstone.com</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=pepperstone</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="L23" s="3" t="inlineStr">
         <is>
           <t>Razor account competitive differentiation and retaining discretionary traders across 15M/1H/4H regimes</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>Pepperstone Razor: AI Pattern Recognition &amp; Reality Cone Copilot</t>
         </is>
       </c>
-      <c r="K23" s="6" t="inlineStr">
+      <c r="N23" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="O23" s="3" t="inlineStr">
         <is>
           <t>High-volume algorithmic and retail traders</t>
         </is>
@@ -1907,7 +2273,7 @@
           <t>Exness</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -1917,42 +2283,57 @@
           <t>Limassol, Cyprus / UK / South Africa</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Exness Terminal (TradingView Web), MetaTrader 4, MetaTrader 5, Exness Trade App</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Web Engine &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Custom REST/WebSocket API into Exness Terminal + Native MT5 Indicator</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>Petr Valov</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Founder</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>partnerships@exness.com</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=exness</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>Empowering high-frequency retail clients with institutional Level 2 resting wall analytics and historical regime search</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>Exness Institutional: Proprietary AI Pattern Matching Engine for Client Portal</t>
         </is>
       </c>
-      <c r="K24" s="6" t="inlineStr">
+      <c r="N24" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>Trillions in monthly volume</t>
         </is>
@@ -1967,7 +2348,7 @@
           <t>Vantage Markets</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -1977,42 +2358,57 @@
           <t>Sydney / Cayman / UK</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5, Vantage App, ProTrader</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Turnkey Client Portal Iframe + TradingView Bridge + MT5 Indicator</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Marc Despallieres</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>Chief Strategy &amp; Trading Officer</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>partners@vantagemarkets.com</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="K25" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Vantage</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr">
         <is>
           <t>Client lifetime value expansion (90 days -&gt; 180+ days) and turnkey web component integration</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>Vantage Markets: Multiplying Client LTV &amp; Lot Turnover with AI Reality Cones</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr">
+      <c r="N25" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="O25" s="3" t="inlineStr">
         <is>
           <t>Aggressive global expansion</t>
         </is>
@@ -2027,7 +2423,7 @@
           <t>ThinkMarkets</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2037,42 +2433,57 @@
           <t>Chicago / London / Australia</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>ThinkTrader (Proprietary TradingView Charts), MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Web Engine &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>ThinkTrader Custom Chart API Integration + MT5 Indicator Package</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Nauman Anees</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Co-Founder</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>partnerships@thinkmarkets.com</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=ThinkMarkets</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr">
         <is>
           <t>ThinkTrader proprietary platform integration and native MT5 indicator distribution</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>ThinkMarkets: AI Volatility Copilot for ThinkTrader &amp; MT5 Desks</t>
         </is>
       </c>
-      <c r="K26" s="6" t="inlineStr">
+      <c r="N26" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>Proprietary trading app + MT5</t>
         </is>
@@ -2087,7 +2498,7 @@
           <t>Tickmill</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2097,42 +2508,57 @@
           <t>London, UK / CySEC / Seychelles</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Tickmill Trader (TradingView Web), MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; Proprietary Web</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Native MT5 EA Indicator + Client Area Web Component</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Illimar Mattus / Sudhanshu Agarwal</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>Co-Founder &amp; Executive Director</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>institutional@tickmill.com</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="K27" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Tickmill</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
         <is>
           <t>Pro account spread revenue maximization and Gold (XAU/USD) volatility forecasting</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>Tickmill Institutional: Proprietary AI Regime Search &amp; Volatility Cones</t>
         </is>
       </c>
-      <c r="K27" s="6" t="inlineStr">
+      <c r="N27" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr">
+      <c r="O27" s="3" t="inlineStr">
         <is>
           <t>Low spread VIP accounts</t>
         </is>
@@ -2147,7 +2573,7 @@
           <t>FP Markets</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2157,42 +2583,57 @@
           <t>Sydney, Australia / CySEC</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5, cTrader, Iress DMA</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Client Portal Turnkey Web Component + MT5 / cTrader Indicator</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Craig Allison</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>partners@fpmarkets.com</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=FPMarkets</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>Iframe client area integration for DMA and raw pricing clients to prevent hesitation in chop</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr">
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>FP Markets: Turnkey Client Portal AI Terminal (Zero Infrastructure Setup)</t>
         </is>
       </c>
-      <c r="K28" s="6" t="inlineStr">
+      <c r="N28" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="O28" s="3" t="inlineStr">
         <is>
           <t>Award-winning Australian ECN</t>
         </is>
@@ -2207,7 +2648,7 @@
           <t>XM Group</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2217,42 +2658,57 @@
           <t>Limassol, Cyprus / Belize / Australia</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 4, MetaTrader 5, XM App (Proprietary)</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader Ecosystem</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Member Area Decision Support Iframe + Native MT5 Indicator</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>Constantinos Cleanthous</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Co-Founder</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>partners@xm.com</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=XM</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t>Educating and empowering 10M+ registered clients with objective statistical boundaries</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>XM Group: Next-Gen AI Decision Support Terminal for Client Area</t>
         </is>
       </c>
-      <c r="K29" s="6" t="inlineStr">
+      <c r="N29" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="O29" s="3" t="inlineStr">
         <is>
           <t>Massive global retail base</t>
         </is>
@@ -2267,7 +2723,7 @@
           <t>Axi</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2277,42 +2733,57 @@
           <t>Sydney, Australia / UK</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5, Axi Copy Trading</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Axi Select Prop Copilot (Web Widget + MT5 EA) + TradingView Script</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Rajesh Yohannan</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>Group CEO</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>partners@axi.com</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Axi</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>Axi Select prop funding ecosystem enhancement with Bayesian Reality Cones</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr">
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>Axi Select: Enhancing Trader Capital Allocation with AI Reality Cones</t>
         </is>
       </c>
-      <c r="K30" s="6" t="inlineStr">
+      <c r="N30" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>Has its own prop incubator Axi Select</t>
         </is>
@@ -2327,7 +2798,7 @@
           <t>FXTM (ForexTime)</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2337,42 +2808,57 @@
           <t>Cyprus / UK / Mauritius</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>MetaTrader 4, MetaTrader 5, FXTM Trader App</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader Ecosystem</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Native MT5 Indicator + MyFXTM Client Area Iframe Widget</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>Olga Rybalkina</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>partners@fxtm.com</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=FXTM</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
         <is>
           <t>Advantage account trader longevity and automated MT5 Reality Cone signals</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>FXTM Advantage: Institutional AI Pattern Matching for Active Clients</t>
         </is>
       </c>
-      <c r="K31" s="6" t="inlineStr">
+      <c r="N31" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="O31" s="3" t="inlineStr">
         <is>
           <t>Emerging market retail powerhouse</t>
         </is>
@@ -2387,7 +2873,7 @@
           <t>BlackBull Markets</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2397,42 +2883,57 @@
           <t>Auckland, New Zealand</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5, cTrader, BlackBull Trade</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; Multi-Platform</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>TradingView Indicator + BlackBull Client Portal Iframe + MT5 EA</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>Michael Walker</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>partners@blackbullmarkets.com</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=BlackBull</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>Institutional liquidity client portal widget with real-time resting iceberg detection</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr">
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>BlackBull Markets: Proprietary AI Reality Cone Integration for MT5 / TradingView</t>
         </is>
       </c>
-      <c r="K32" s="6" t="inlineStr">
+      <c r="N32" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>TradingView broker partner</t>
         </is>
@@ -2447,7 +2948,7 @@
           <t>AvaTrade</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2457,42 +2958,57 @@
           <t>Dublin, Ireland / ASIC / FSCA</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>AvaTradeGO (Proprietary), WebTrader, MetaTrader 4, MetaTrader 5, AvaOptions</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Web Engine &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>AvaProtect Complementary Volatility API + WebTrader Embed</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Dáire Ferguson</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>partners@avatrade.com</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="K33" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=AvaTrade</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>AvaProtect risk management suite augmentation with predictive volatility envelopes</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr">
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>AvaProtect x XPredictor: Next-Gen Empirical Risk Boundaries for AvaTrade Clients</t>
         </is>
       </c>
-      <c r="K33" s="6" t="inlineStr">
+      <c r="N33" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="O33" s="3" t="inlineStr">
         <is>
           <t>Strong retail risk products</t>
         </is>
@@ -2507,7 +3023,7 @@
           <t>Eightcap</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2517,42 +3033,57 @@
           <t>Melbourne, Australia / Bahamas</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; MetaTrader</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>TradingView Integration + MT5 Indicator for Institutional Prop Partners</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>Joel Murphy</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>partners@eightcap.com</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="K34" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Eightcap</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="L34" s="3" t="inlineStr">
         <is>
           <t>Prop firm liquidity provider integration and high-volume crypto/CFD analytics</t>
         </is>
       </c>
-      <c r="J34" s="3" t="inlineStr">
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>Eightcap Partner Desk: Institutional AI Reality Cones for Prop &amp; Retail Traders</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr">
+      <c r="N34" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>Major prop trading infrastructure broker</t>
         </is>
@@ -2567,7 +3098,7 @@
           <t>OANDA</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2577,42 +3108,57 @@
           <t>New York, USA / London / Singapore</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>TradingView, OANDA Trade (Proprietary Web/Mobile), MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>TradingView Partner &amp; Proprietary Web</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>TradingView Integration + OANDA Prop Trader Risk Copilot Web Widget</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>Gavin Bambury</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>institutional@oanda.com</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="K35" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=OANDA</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="L35" s="3" t="inlineStr">
         <is>
           <t>OANDA Prop Trader and API client retention with institutional Bayesian modeling</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr">
+      <c r="M35" s="3" t="inlineStr">
         <is>
           <t>OANDA Prop Trader: Institutional AI Pattern Recognition &amp; Reality Cones</t>
         </is>
       </c>
-      <c r="K35" s="6" t="inlineStr">
+      <c r="N35" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L35" s="3" t="inlineStr">
+      <c r="O35" s="3" t="inlineStr">
         <is>
           <t>Recently launched OANDA Prop Trader</t>
         </is>
@@ -2627,7 +3173,7 @@
           <t>CMC Markets</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2637,42 +3183,57 @@
           <t>London, UK (FTSE 250)</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>NextGen (Proprietary Platform), MetaTrader 4</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Institutional Platform</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>NextGen Custom API / White-Label Institutional Web Component</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>Peter Cruddas</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Founder</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>institutional@cmcmarkets.com</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="K36" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=CMCMarkets</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="L36" s="3" t="inlineStr">
         <is>
           <t>NextGen platform institutional add-on for sovereign desks and high-net-worth traders</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr">
+      <c r="M36" s="3" t="inlineStr">
         <is>
           <t>CMC Markets Connect: Proprietary AI Regime Search for Institutional Desks</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr">
+      <c r="N36" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="O36" s="3" t="inlineStr">
         <is>
           <t>Tier-1 institutional broker</t>
         </is>
@@ -2687,7 +3248,7 @@
           <t>Saxo Bank</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Investment Bank</t>
         </is>
@@ -2697,42 +3258,57 @@
           <t>Copenhagen, Denmark / Global</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>SaxoTraderGO (Proprietary Web), SaxoTraderPRO (Desktop)</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Institutional Platform</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Saxo OpenAPI Headless Integration + Dedicated Institutional Web Component</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>Kim Fournais</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>CEO &amp; Founder</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>institutional@saxobank.com</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=SaxoBank</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
+      <c r="L37" s="3" t="inlineStr">
         <is>
           <t>OpenAPI integration for institutional wealth and active multi-asset trading desks</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr">
+      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>Saxo Bank Institutional: OpenAPI Historical Regime Search &amp; Volatility Cones</t>
         </is>
       </c>
-      <c r="K37" s="6" t="inlineStr">
+      <c r="N37" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L37" s="3" t="inlineStr">
+      <c r="O37" s="3" t="inlineStr">
         <is>
           <t>Global banking infrastructure</t>
         </is>
@@ -2747,7 +3323,7 @@
           <t>Swissquote</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Banking &amp; FX Broker</t>
         </is>
@@ -2757,42 +3333,57 @@
           <t>Gland, Switzerland (SIX:SQN)</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Advanced Trader (Proprietary), MetaTrader 4, MetaTrader 5, FIX API</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Institutional Platform &amp; MT5</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Swissquote eForex Portal Embed + Native MT5 EA</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>Marc Bürki</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>institutional@swissquote.ch</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="K38" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Swissquote</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="L38" s="3" t="inlineStr">
         <is>
           <t>Swiss-grade quantitative analytics for tier-1 asset managers and active CFD traders</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr">
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>Swissquote Institutional: Proprietary AI Reality Cone Engine for eForex Desks</t>
         </is>
       </c>
-      <c r="K38" s="6" t="inlineStr">
+      <c r="N38" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L38" s="3" t="inlineStr">
+      <c r="O38" s="3" t="inlineStr">
         <is>
           <t>Swiss banking safety reputation</t>
         </is>
@@ -2807,7 +3398,7 @@
           <t>Admirals</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2817,42 +3408,57 @@
           <t>Tallinn, Estonia / UK / CySEC</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Admirals Platform (TradingView Web), MetaTrader 4, MetaTrader 5</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; Proprietary Web</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>MT5 'Supreme Edition' AI Add-on Module + WebTrader Embed</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Sergei Bogatenkov</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>partners@admiralmarkets.com</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=Admirals</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="L39" s="3" t="inlineStr">
         <is>
           <t>Supreme Edition MT5 plugin upgrade with AI-powered historical pattern matching</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr">
+      <c r="M39" s="3" t="inlineStr">
         <is>
           <t>Admirals Supreme Edition: Integrating AI Reality Cones for Active Clients</t>
         </is>
       </c>
-      <c r="K39" s="6" t="inlineStr">
+      <c r="N39" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L39" s="3" t="inlineStr">
+      <c r="O39" s="3" t="inlineStr">
         <is>
           <t>Famous for MT5 Supreme Edition</t>
         </is>
@@ -2867,7 +3473,7 @@
           <t>RoboForex</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>FX/CFD Broker</t>
         </is>
@@ -2877,42 +3483,57 @@
           <t>Belize / CySEC</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>R StocksTrader (TradingView Web), MetaTrader 4, MetaTrader 5, cTrader</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>MetaTrader &amp; Modern Web</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>R StocksTrader Iframe Widget + Native MT5 EA Indicator</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>Partnerships Desk</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>Head of Business Development</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>partners@roboforex.com</t>
         </is>
       </c>
-      <c r="H40" s="5" t="inlineStr">
+      <c r="K40" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=RoboForex</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr">
+      <c r="L40" s="3" t="inlineStr">
         <is>
           <t>Prime and ECN account client retention and automated Telegram signal bot integration</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr">
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>RoboForex ECN: Turnkey AI Reality Cone Copilot &amp; Automated Signal Engine</t>
         </is>
       </c>
-      <c r="K40" s="6" t="inlineStr">
+      <c r="N40" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L40" s="3" t="inlineStr">
+      <c r="O40" s="3" t="inlineStr">
         <is>
           <t>Huge international affiliate reach</t>
         </is>
@@ -2927,7 +3548,7 @@
           <t>IG Group</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="9" t="inlineStr">
         <is>
           <t>Multi-Asset Broker</t>
         </is>
@@ -2937,42 +3558,57 @@
           <t>London, UK (FTSE 250)</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>IG Trading Platform (Proprietary), MetaTrader 4, ProRealTime, L2 Dealer</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Proprietary Institutional Platform</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>IG Institutional REST API / Web Component + ProRealTime Indicator</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>Charlie Rozes / Matt Macklin</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>Executive Leadership</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>institutional@ig.com</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="K41" s="7" t="inlineStr">
         <is>
           <t>https://aravinthragav.github.io/xpredictor/?partner=IG</t>
         </is>
       </c>
-      <c r="I41" s="3" t="inlineStr">
+      <c r="L41" s="3" t="inlineStr">
         <is>
           <t>Premium client retention during macroeconomic consolidation and institutional Gold/Index analytics</t>
         </is>
       </c>
-      <c r="J41" s="3" t="inlineStr">
+      <c r="M41" s="3" t="inlineStr">
         <is>
           <t>IG Prime: Institutional AI Pattern Search &amp; Bayesian Volatility Cones</t>
         </is>
       </c>
-      <c r="K41" s="6" t="inlineStr">
+      <c r="N41" s="8" t="inlineStr">
         <is>
           <t>Ready for Outreach</t>
         </is>
       </c>
-      <c r="L41" s="3" t="inlineStr">
+      <c r="O41" s="3" t="inlineStr">
         <is>
           <t>Global spread betting &amp; CFD leader</t>
         </is>
@@ -2980,52 +3616,235 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Platform Archetype</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Representative Partners</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>How They Trade / Chart</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>XPredictor Integration Package</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Key Value Pitch to Partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="55" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>1. MetaTrader Ecosystem (MT5 / MT4)</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>FTMO, IC Markets, Exness, Fidelcrest, The 5%ers, Pepperstone</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Desktop C++ terminal (MQL5/MQL4) + Mobile. High volume algorithmic and discretionary EAs.</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Native MetaTrader 5 Indicator (.mq5) + Expert Advisor Signal Copilot + Client Portal Web Iframe</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Zero-latency desktop chart overlay. Traders drop it directly into MT5 without installing third-party apps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>2. Modern Web Prop Stack (TradeLocker, DXtrade, Match-Trader)</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>FundedNext, Funding Pips, Blue Guardian, MyFundedFX, Goat Funded Trader</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Web-first trading dashboards with TradingView charting library. Popularized after MetaQuotes prop crackdowns.</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Turnkey Client Portal Web Component / Iframe (&lt;iframe src='...'&gt;) + Webhook Signals</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>3-minute zero-development deployment directly in their React/Vue CRM or trader dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>3. TradingView Partner Brokers</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Pepperstone, IC Markets, BlackBull Markets, Vantage, Eightcap, OANDA</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Traders trade directly from TradingView charts or broker web interfaces powered by TradingView.</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>TradingView Pine Script Tool + Webhook Signal Dispatcher + Co-Branded Web Terminal</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Enhances their TradingView brand equity. Gives traders proprietary predictive cones directly where they chart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>4. US Futures Stack (Tradovate / NinjaTrader)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Topstep, Apex Trader Funding, Fast Track Trading</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Rithmic / CQG tick feeds + NinjaTrader (C# NinjaScript) and Tradovate cloud platform.</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>NinjaTrader 8 C# Add-on Indicator (.cs) + Tradovate Browser Risk Extension Overlay</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Guards against intraday trailing drawdown blowups during CPI/FOMC futures spikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>5. Proprietary Institutional Web Engines</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Saxo Bank (SaxoTraderGO), CMC Markets (NextGen), ThinkMarkets (ThinkTrader), IG Group</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Proprietary in-house institutional trading engines and custom REST/OpenAPI architectures.</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Headless REST / WebSocket API Gateway + Enterprise Co-Branded Standalone Terminal</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Enriches their proprietary platform with high-margin quantitative AI analytics without revealing proprietary code.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3039,24 +3858,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Template Name</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Cold Outreach Email Copy</t>
         </is>
       </c>
     </row>
     <row r="2" ht="220" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>SEQUENCE 1: FOR PROP TRADING FIRMS (CEOs, Heads of Risk)</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Subject: {{firm_name}} x XPredictor: Dynamic Max Drawdown &amp; Reality Cone Copilot
 Hi {{first_name}},
@@ -3064,7 +3883,7 @@
 We've engineered XPredictor (https://aravinthragav.github.io/xpredictor/?partner={{partner_key}}), a proprietary institutional AI pattern matching engine that gives your evaluation and funded traders an empirical Risk Copilot:
 1. Continuous Bayesian Reality Cones: Visualizes mathematically probable price bounds (±2.1σ, Mean E[P]) over the forward 22 bars, warning traders before they breach drawdown limits.
 2. 50M+ Historical Regime Analogs: Sub-35ms pattern retrieval matching current price action against historical setups (Zero Lookahead Bias).
-3. Turnkey Integration: Deploys directly into your Client Portal via a 3-minute iframe, or native MT5 desktop indicator (.mq5).
+3. Turnkey Integration for {{supported_software}}: Deploys directly into your Client Portal via a 3-minute iframe, or native MT5 desktop indicator (.mq5).
 We've provisioned a live co-branded sandbox for {{firm_name}} here: https://aravinthragav.github.io/xpredictor/?partner={{partner_key}}
 Would you be open to a 10-minute demo on how this extends funded account lifespan by 3.2x?
 Best regards,
@@ -3075,12 +3894,12 @@
       </c>
     </row>
     <row r="3" ht="220" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>SEQUENCE 2: FOR FX / CFD BROKERS (CCOs, Heads of Brokerage)</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Subject: {{firm_name}} Client Area: Embeddable AI Reality Cone Terminal &amp; 18x Lot ROI
 Hi {{first_name}},
@@ -3088,8 +3907,8 @@
 We built XPredictor to solve trader chop hesitation by providing institutional AI historical regime matching and forward Bayesian volatility boundaries directly inside your Client Portal.
 Key Broker Commercial Highlights:
 • Volume Multiplier: Keeping just 500 active traders from quitting chop adds an estimated $180,000+ in annual spread revenue (18x partner ROI).
+• Tailored for {{supported_software}}: Plugs into your existing platform stack without infrastructure changes.
 • 100% Non-Advisory: Classified as objective volatility and historical charting analytics (like Bollinger Bands / ATR), eliminating regulatory friction.
-• Zero Development Burden: Single embeddable iframe / web component requiring zero changes to your core MT5 bridge.
 See your live co-branded partner sandbox: https://aravinthragav.github.io/xpredictor/?partner={{partner_key}}
 Can we set up a brief 10-minute call this Thursday or Friday to show you the partner economics?
 Best regards,
@@ -3100,12 +3919,12 @@
       </c>
     </row>
     <row r="4" ht="220" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>SEQUENCE 3: THE 3-DAY FOLLOW-UP (SHORT &amp; PUNCHY)</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Subject: Re: {{firm_name}} x XPredictor Sandbox
 Hi {{first_name}},
@@ -3122,7 +3941,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3137,24 +3956,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Funnel Stage</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Target Count</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Description / Benchmark</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Total Verified Targets</t>
         </is>
@@ -3171,7 +3990,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Target Open Rate</t>
         </is>
@@ -3188,7 +4007,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Target Reply Rate</t>
         </is>
@@ -3205,7 +4024,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Target Pilot Demos</t>
         </is>
@@ -3222,7 +4041,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>30-Day Pilots Signed</t>
         </is>
@@ -3239,7 +4058,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Contract Target</t>
         </is>

</xml_diff>